<commit_message>
Added Bill Payment Test Cases
</commit_message>
<xml_diff>
--- a/TestData/ViewFundsTransfers.xlsx
+++ b/TestData/ViewFundsTransfers.xlsx
@@ -3,13 +3,13 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1884" yWindow="1884" windowWidth="17280" windowHeight="8880" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="162913" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -390,160 +390,141 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="B1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
+    <row r="1">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>243</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>669</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>667</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>30000</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Tue Jun 02 2026 16:27:56 GMT+0530 (India Standard Time)</t>
+        </is>
+      </c>
+    </row>
     <row r="2">
       <c r="B2" t="inlineStr">
         <is>
-          <t>243</t>
+          <t>119</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>669</t>
+          <t>115</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>128</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>30000</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Tue Jun 02 2026 16:27:56 GMT+0530 (India Standard Time)</t>
+          <t>Fri Aug 16 2024 13:02:15 GMT+0530 (India Standard Time)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="B3" t="inlineStr">
         <is>
-          <t>119</t>
+          <t>106</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>115</t>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>21</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>9</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Fri Aug 16 2024 13:02:15 GMT+0530 (India Standard Time)</t>
+          <t>Wed Aug 14 2024 20:39:26 GMT+0530 (India Standard Time)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="B4" t="inlineStr">
         <is>
-          <t>106</t>
+          <t>74</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>40000</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Wed Aug 14 2024 20:39:26 GMT+0530 (India Standard Time)</t>
+          <t>Sun Aug 11 2024 14:28:07 GMT+0530 (India Standard Time)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="B5" t="inlineStr">
         <is>
-          <t>74</t>
+          <t>24</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>91</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>83</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>40000</t>
+          <t>10000</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Sun Aug 11 2024 14:28:07 GMT+0530 (India Standard Time)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>91</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>10000</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
           <t>Sat Aug 10 2024 23:24:00 GMT+0530 (India Standard Time)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>91</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>83</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>83</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>115</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>115</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>128</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>128</t>
         </is>
       </c>
     </row>

</xml_diff>